<commit_message>
test: add real order parser fixtures
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체 로드맵" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현재 상태" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검증 체크리스트" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류·제외 기능" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다음 작업" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="전체 로드맵" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="현재 상태" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="검증 체크리스트" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="보류·제외 기능" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="다음 작업" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +77,12 @@
     <font>
       <name val="Malgun Gothic"/>
       <b val="1"/>
+      <color rgb="001D5A99"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Malgun Gothic"/>
+      <b val="1"/>
       <color rgb="008A6D11"/>
       <sz val="10"/>
     </font>
@@ -93,7 +99,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +114,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E3F2E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EDF9"/>
       </patternFill>
     </fill>
     <fill>
@@ -152,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -185,13 +196,16 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -586,7 +600,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -843,17 +856,17 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>잠금이 진짜 잠기는지 확인 — 회사/멤버 row 확인, 타 회사 접근 차단 실측</t>
+          <t>잠금이 진짜 잠기는지 확인 — 회사/멤버 row, anon 차단, policy 확인 완료. 타 계정 A/B 격리 실측만 남음</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>다음</t>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>supabase-rls-policy §9 시나리오</t>
+          <t>회사 row·owner 멤버·anon 차단·policy 존재 확인(2026-07-02)</t>
         </is>
       </c>
     </row>
@@ -873,7 +886,7 @@
           <t>실제 주문 장부 저장 — 새로고침해도 주문이 남고, 거래처별 일/월 합계가 나옴</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -900,7 +913,7 @@
           <t>저장된 장부에서 합산표·명세서를 다시 꺼내 쓰기(재출력)</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -927,7 +940,7 @@
           <t>지금은 일부러 안 만드는 것들(아래 보류/제외 표 참조)</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>제외/2차</t>
         </is>
@@ -953,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -975,7 +988,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1079,87 +1091,104 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>8a-검증(부분 완료)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>회사/멤버 row(히든식품·owner) 확인, 비로그인(anon) 조회 차단 확인([]), RLS policy 존재 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>주문 DB 저장</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>주문 확정해도 아직 브라우저 메모리에만 있음(새로고침하면 사라짐)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>주문 목록 DB 조회</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>저장된 장부에서 주문 목록 불러오기</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>합산표 DB 연결</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>저장된 주문으로 합산표 만들기</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>거래명세서 DB 재출력</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>지난 주문의 명세서를 언제든 다시 인쇄</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>RLS A/B 회사 격리 실측</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>다른 회사 계정으로 내 데이터가 진짜 안 보이는지 실제 확인</t>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>타 계정/타 회사(B)로 히든식품(A) 데이터가 진짜 안 보이는지 실측 — 8a-검증의 마지막 남은 항목</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1200,7 +1229,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1229,7 +1257,7 @@
           <t>옛 정적 데모 회귀 테스트</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>✅ 통과 5/5</t>
         </is>
@@ -1246,7 +1274,7 @@
           <t>앱 계산/파싱/합산 자동 테스트</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>✅ 통과 32/32</t>
         </is>
@@ -1263,7 +1291,7 @@
           <t>배포용 빌드가 깨지지 않는지</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1280,7 +1308,7 @@
           <t>알려진 보안 취약점 검사</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>✅ 0건</t>
         </is>
@@ -1297,7 +1325,7 @@
           <t>비밀키가 저장소에 안 올라가는지</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>✅ 확인(미추적)</t>
         </is>
@@ -1314,7 +1342,7 @@
           <t>장부 테이블/잠금/회사생성 함수 설치</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>✅ 적용 성공</t>
         </is>
@@ -1331,7 +1359,7 @@
           <t>이메일 매직링크로 입장</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1348,7 +1376,7 @@
           <t>'히든식품' 회사 등록</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1365,7 +1393,7 @@
           <t>로그인+회사 후 앱 화면 진입</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1374,17 +1402,68 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>RLS 실측</t>
+          <t>Supabase 회사/멤버 row 확인</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>타 회사 데이터 차단 실제 확인</t>
+          <t>장부에 회사가 진짜 기록됐는지 SQL로 확인</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>⏳ 미실측 — 다음(8a-검증)</t>
+          <t>✅ 성공 — 히든식품 / role=owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>비로그인(anon) 조회 차단</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>로그인 없이 공개 키로 회사 데이터가 보이는지</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>✅ 차단 확인 — [] 반환</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>RLS policy 존재 확인</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>ordermoa_* 테이블마다 잠금 규칙이 설치됐는지</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>✅ 확인 — 테이블별 policy 존재</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>타 계정 A/B 회사 격리 실측</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>다른 계정/다른 회사로 히든식품 데이터 차단 확인</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>⏳ 미실측 — 8a-검증 남은 항목</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1504,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1449,7 +1527,7 @@
           <t>미수금/입금 본격 관리</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1466,7 +1544,7 @@
           <t>세금계산서 발행(홈택스)</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1483,7 +1561,7 @@
           <t>PDF 파일 생성</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1500,7 +1578,7 @@
           <t>OCR/사진 인식</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
@@ -1517,7 +1595,7 @@
           <t>카카오톡 자동 읽기</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
@@ -1534,7 +1612,7 @@
           <t>이카운트 연동</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
@@ -1551,7 +1629,7 @@
           <t>매입처별 발주 저장/기본 매입처</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1568,7 +1646,7 @@
           <t>정확한 회계 마진(원가/재고/세무)</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1585,7 +1663,7 @@
           <t>단가 변경 이력</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1602,7 +1680,7 @@
           <t>직원 권한 UI(staff)</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1619,7 +1697,7 @@
           <t>거래처 주문 링크</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
@@ -1669,7 +1747,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1698,32 +1775,32 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>8a-검증</t>
+          <t>8a-검증 마무리</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Supabase 실측 검증</t>
+          <t>타 계정 A/B 회사 격리 실측</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>히든식품 회사/멤버 row 실제 확인 + RLS 기본 확인(타 계정 차단). 8b에서 주문을 저장하기 전에 잠금이 진짜 잠기는지 먼저 확인해야 안전.</t>
+          <t>회사 row·anon 차단·policy 존재는 확인 완료. 남은 건 두 번째 계정(B회사)으로 로그인해 히든식품(A) 데이터가 select 0행/insert 거부되는지 실측하는 것뿐. 이것까지 되면 잠금 검증 끝.</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>짧음(30분~1시간)</t>
+          <t>짧음(30분 내)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="16" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1748,7 +1825,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="n">
+      <c r="A7" s="16" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: add order persistence foundation and admin dashboard
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,12 +77,6 @@
     <font>
       <name val="Malgun Gothic"/>
       <b val="1"/>
-      <color rgb="001D5A99"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Malgun Gothic"/>
-      <b val="1"/>
       <color rgb="008A6D11"/>
       <sz val="10"/>
     </font>
@@ -99,7 +93,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -114,11 +108,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E3F2E5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EDF9"/>
       </patternFill>
     </fill>
     <fill>
@@ -163,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -196,16 +185,10 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -844,9 +827,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>8a-검증  ◀ 현재 위치</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>8a-검증</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -856,24 +839,24 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>잠금이 진짜 잠기는지 확인 — 회사/멤버 row, anon 차단, policy 확인 완료. 타 계정 A/B 격리 실측만 남음</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+          <t>잠금이 진짜 잠기는지 확인 완료 — 회사/멤버 row·anon 차단·policy 존재 + A/B 격리(0/0/0)·위조 insert 거부</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>회사 row·owner 멤버·anon 차단·policy 존재 확인(2026-07-02)</t>
+          <t>A/B 격리 실측 통과(2026-07-02)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>단위 8b</t>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>단위 8b  ◀ 현재 위치</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -886,7 +869,7 @@
           <t>실제 주문 장부 저장 — 새로고침해도 주문이 남고, 거래처별 일/월 합계가 나옴</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -913,7 +896,7 @@
           <t>저장된 장부에서 합산표·명세서를 다시 꺼내 쓰기(재출력)</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -940,7 +923,7 @@
           <t>지금은 일부러 안 만드는 것들(아래 보류/제외 표 참조)</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>제외/2차</t>
         </is>
@@ -966,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1098,17 +1081,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>8a-검증(부분 완료)</t>
+          <t>8a-검증(완료)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>회사/멤버 row(히든식품·owner) 확인, 비로그인(anon) 조회 차단 확인([]), RLS policy 존재 확인</t>
+          <t>회사/멤버 row·anon 차단·policy 확인 + A/B 격리(다른 회사 사용자엔 회사/멤버/거래처 0/0/0)·위조 insert 거부(RLS 42501)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -1125,7 +1108,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -1142,7 +1125,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -1159,7 +1142,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>다음</t>
         </is>
@@ -1172,23 +1155,6 @@
       <c r="C14" s="6" t="inlineStr">
         <is>
           <t>지난 주문의 명세서를 언제든 다시 인쇄</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>다음</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>RLS A/B 회사 격리 실측</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>타 계정/타 회사(B)로 히든식품(A) 데이터가 진짜 안 보이는지 실측 — 8a-검증의 마지막 남은 항목</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1257,7 +1223,7 @@
           <t>옛 정적 데모 회귀 테스트</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>✅ 통과 5/5</t>
         </is>
@@ -1274,7 +1240,7 @@
           <t>앱 계산/파싱/합산 자동 테스트</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>✅ 통과 32/32</t>
         </is>
@@ -1291,7 +1257,7 @@
           <t>배포용 빌드가 깨지지 않는지</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1308,7 +1274,7 @@
           <t>알려진 보안 취약점 검사</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>✅ 0건</t>
         </is>
@@ -1325,7 +1291,7 @@
           <t>비밀키가 저장소에 안 올라가는지</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>✅ 확인(미추적)</t>
         </is>
@@ -1342,7 +1308,7 @@
           <t>장부 테이블/잠금/회사생성 함수 설치</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>✅ 적용 성공</t>
         </is>
@@ -1359,7 +1325,7 @@
           <t>이메일 매직링크로 입장</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1376,7 +1342,7 @@
           <t>'히든식품' 회사 등록</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1393,7 +1359,7 @@
           <t>로그인+회사 후 앱 화면 진입</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>✅ 성공</t>
         </is>
@@ -1410,7 +1376,7 @@
           <t>장부에 회사가 진짜 기록됐는지 SQL로 확인</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>✅ 성공 — 히든식품 / role=owner</t>
         </is>
@@ -1427,7 +1393,7 @@
           <t>로그인 없이 공개 키로 회사 데이터가 보이는지</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>✅ 차단 확인 — [] 반환</t>
         </is>
@@ -1444,7 +1410,7 @@
           <t>ordermoa_* 테이블마다 잠금 규칙이 설치됐는지</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>✅ 확인 — 테이블별 policy 존재</t>
         </is>
@@ -1453,17 +1419,34 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>타 계정 A/B 회사 격리 실측</t>
+          <t>A/B 회사 격리 select 실측</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>다른 계정/다른 회사로 히든식품 데이터 차단 확인</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>⏳ 미실측 — 8a-검증 남은 항목</t>
+          <t>다른 회사 사용자엔 히든식품 데이터가 안 보이는지</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>✅ 성공 — 회사/멤버/거래처 0/0/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>A회사 위조 insert 차단</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>다른 회사 사용자가 히든식품에 몰래 넣기 시도</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>✅ 차단 성공 — RLS 오류 42501</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1510,7 @@
           <t>미수금/입금 본격 관리</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1544,7 +1527,7 @@
           <t>세금계산서 발행(홈택스)</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1561,7 +1544,7 @@
           <t>PDF 파일 생성</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1578,7 +1561,7 @@
           <t>OCR/사진 인식</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
@@ -1595,7 +1578,7 @@
           <t>카카오톡 자동 읽기</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
@@ -1612,7 +1595,7 @@
           <t>이카운트 연동</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
@@ -1629,7 +1612,7 @@
           <t>매입처별 발주 저장/기본 매입처</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1646,7 +1629,7 @@
           <t>정확한 회계 마진(원가/재고/세무)</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1663,7 +1646,7 @@
           <t>단가 변경 이력</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1680,7 +1663,7 @@
           <t>직원 권한 UI(staff)</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
@@ -1697,7 +1680,7 @@
           <t>거래처 주문 링크</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
@@ -1723,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1775,75 +1758,50 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="14" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>8a-검증 마무리</t>
+          <t>8b</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>타 계정 A/B 회사 격리 실측</t>
+          <t>주문 저장/조회/기간 집계</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>회사 row·anon 차단·policy 존재는 확인 완료. 남은 건 두 번째 계정(B회사)으로 로그인해 히든식품(A) 데이터가 select 0행/insert 거부되는지 실측하는 것뿐. 이것까지 되면 잠금 검증 끝.</t>
+          <t>8a-검증(잠금)이 전부 통과돼 이제 안전하게 데이터를 쌓을 수 있다. 핵심 가치가 '기록이 남는다'로 완성되는 단계. 주문 확정→ordermoa_orders/items 저장→새로고침 후에도 유지.</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>짧음(30분 내)</t>
+          <t>중간(1세션)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>8b</t>
+          <t>8c</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>주문 저장/조회/기간 집계</t>
+          <t>합산표/거래명세서 DB 연결</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>핵심 가치가 '기록이 남는다'로 완성되는 단계. 주문 확정→ordermoa_orders/items 저장→새로고침 후에도 유지.</t>
+          <t>저장된 주문으로 합산표·명세서 재출력. 8b 위에 얹는 조회 작업.</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>중간(1세션)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>8c</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>합산표/거래명세서 DB 연결</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>저장된 주문으로 합산표·명세서 재출력. 8b 위에 얹는 조회 작업.</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>중간</t>
         </is>

</xml_diff>

<commit_message>
feat: add customer management and supplier persistence
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작업보드" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="완료된 기반" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검증 체크리스트" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외 기능" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="요약" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="작업보드" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="완료된 기반" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="검증 체크리스트" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="제외 기능" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -94,6 +99,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -536,7 +544,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>기준정보 관리 1차 (거래처/품목·별칭/단가 CRUD) + 매입처 DB화 설계 승인</t>
+          <t>W02 거래처 관리 CRUD 완료. W05/W06 매입처 DB화 코드·마이그레이션 준비 완료, Supabase 적용 실측 대기.</t>
         </is>
       </c>
     </row>
@@ -560,7 +568,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 16개 — 완료 1 · 다음 12 · 보류 3</t>
+          <t>총 16개 — 완료 2 · 다음 9 · 진행 중 2 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -587,7 +595,8 @@
           <t>fc59baa docs: add ordermoa system planning charter
 a97dca8 feat: add inline product creation from unmatched orders
 8d95da6 feat: refine supplier purchase selection progress
-490ca0b feat: add product search and supplier purchase grouping</t>
+490ca0b feat: add product search and supplier purchase grouping
+34d30df docs: refine ordermoa roadmap progress board</t>
         </is>
       </c>
     </row>
@@ -724,9 +733,9 @@
           <t>기준정보 CRUD — 거래처 관리</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -736,7 +745,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>가람식당 같은 거래처(파는 곳)를 사용자가 직접 추가·수정·보관하는 화면. 지금은 샘플 5곳이 박혀 있어 못 고칩니다.</t>
+          <t>가람식당 같은 거래처(파는 곳)를 사용자가 직접 추가·수정·보관하는 화면. 데모 모드와 Supabase 모드 저장 로직을 모두 연결했습니다.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -751,7 +760,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>거래처 추가→새로고침 후 유지, 수정 반영, 보관(숨김) 동작. web npm test + build 통과.</t>
+          <t>거래처 추가/수정/보관 화면 구현. web npm test 83/83 + build 통과. Supabase 실사용 새로고침 확인은 다음 현장 실측에서 진행.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -871,9 +880,9 @@
           <t>매입처 DB화 — suppliers 테이블 설계</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -883,7 +892,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>야채매입처 같은 매입처(사 오는 곳)를 DB에 정식 저장하는 설계. 지금은 화면에만 있어서 새로고침하면 매입처 지정이 사라질 수 있습니다.</t>
+          <t>야채매입처 같은 매입처(사 오는 곳)를 DB에 정식 저장하는 마이그레이션을 준비했습니다. Supabase SQL 적용과 RLS 실측만 남았습니다.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -893,12 +902,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Codex 마이그레이션 승인 (ordermoa_suppliers + RLS + 교차회사 트리거 + unique 이름).</t>
+          <t>0004_suppliers.sql을 Supabase SQL Editor에서 적용.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>마이그레이션 적용 후 RLS A/B 격리 확인, 테이블 생성 확인.</t>
+          <t>마이그레이션 파일 작성, RLS/교차회사 트리거 포함, web npm test 83/83 + build 통과. 실제 Supabase 적용 후 테이블/RLS 확인 필요.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -920,9 +929,9 @@
           <t>매입처 DB화 — 품목별 기본 매입처 연결</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -932,7 +941,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>품목마다 '이건 야채매입처에서 산다'를 DB에 저장(products에 매입처 연결 컬럼 추가). 신규 품목 즉석 등록의 기본 매입처도 진짜 저장됩니다.</t>
+          <t>품목마다 '이건 야채매입처에서 산다'를 DB에 저장하는 코드 연결을 넣었습니다. 신규 품목 즉석 등록의 기본 매입처도 DB에 저장되도록 준비했습니다.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -947,7 +956,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>품목의 매입처 지정→F5 후 유지→합산표 매입처별 문장에 반영. 테스트+빌드 통과.</t>
+          <t>시드 보충/품목 매입처 연결 테스트 추가. web npm test 83/83 + build 통과. Supabase 0004 적용 후 F5 유지 실측 필요.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1305,7 +1314,7 @@
           <t>인쇄/명세서 양식 보정</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
@@ -1352,7 +1361,7 @@
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
@@ -1399,7 +1408,7 @@
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
@@ -1610,12 +1619,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>파서/합산/검색/주문 저장 빌더 자동 테스트</t>
+          <t>파서/합산/검색/주문 저장 빌더/거래처·매입처 보강 자동 테스트</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>통과 78/78</t>
+          <t>통과 83/83</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: capture feedback roadmap after db validation
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,11 +63,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
@@ -84,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -99,9 +94,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -544,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W02 거래처 관리 CRUD 완료. W05/W06 매입처 DB화 코드·마이그레이션 준비 완료, Supabase 적용 실측 대기.</t>
+          <t>W05/W06/W08 실측 완료(0004 적용 + 비밀번호 로그인 + 주문 저장 F5 유지). 다음: W17 합산표 개선 팩(발주 문장 템플릿·누락 검수·색상) → W07 매입처 관리 → W03 품목·별칭.</t>
         </is>
       </c>
     </row>
@@ -568,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 16개 — 완료 2 · 다음 9 · 진행 중 2 · 보류 3</t>
+          <t>총 17개 — 완료 5 · 다음 9 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -592,11 +584,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>fc59baa docs: add ordermoa system planning charter
-a97dca8 feat: add inline product creation from unmatched orders
-8d95da6 feat: refine supplier purchase selection progress
-490ca0b feat: add product search and supplier purchase grouping
-34d30df docs: refine ordermoa roadmap progress board</t>
+          <t>a696a36 feat: add password login fallback
+38f4e6c fix: harden supplier migration guidance
+7d3de93 feat: add customer management and supplier persistence
+34d30df docs: refine ordermoa roadmap progress board
+fc59baa docs: add ordermoa system planning charter</t>
         </is>
       </c>
     </row>
@@ -611,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -880,9 +872,9 @@
           <t>매입처 DB화 — suppliers 테이블 설계</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -892,7 +884,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>야채매입처 같은 매입처(사 오는 곳)를 DB에 정식 저장하는 마이그레이션을 준비했습니다. Supabase SQL 적용과 RLS 실측만 남았습니다.</t>
+          <t>야채매입처 같은 매입처(사 오는 곳)를 DB에 정식 저장하는 보관함을 만들었습니다. 2026-07-07 Supabase에 적용 완료.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -902,12 +894,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0004_suppliers.sql을 Supabase SQL Editor에서 적용.</t>
+          <t>완료 — 0004_suppliers.sql Supabase 적용됨.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>마이그레이션 파일 작성, RLS/교차회사 트리거 포함, web npm test 83/83 + build 통과. 실제 Supabase 적용 후 테이블/RLS 확인 필요.</t>
+          <t>2026-07-07 사용자가 SQL Editor에서 적용, Table Editor에서 ordermoa_suppliers 테이블 확인. RLS 4정책+교차회사 트리거 포함.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -929,9 +921,9 @@
           <t>매입처 DB화 — 품목별 기본 매입처 연결</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -941,7 +933,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>품목마다 '이건 야채매입처에서 산다'를 DB에 저장하는 코드 연결을 넣었습니다. 신규 품목 즉석 등록의 기본 매입처도 DB에 저장되도록 준비했습니다.</t>
+          <t>품목마다 '이건 야채매입처에서 산다'가 DB에 저장됩니다. 신규 품목 즉석 등록의 기본 매입처도 함께 저장됩니다.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -951,12 +943,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>W05(테이블) 적용 완료.</t>
+          <t>완료 — W05 적용과 함께 동작.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>시드 보충/품목 매입처 연결 테스트 추가. web npm test 83/83 + build 통과. Supabase 0004 적용 후 F5 유지 실측 필요.</t>
+          <t>2026-07-07 실측: 로그인 후 샘플 시드에 매입처 포함 설치, 주문·화면 F5 후 유지 확인. web npm test 83/83 + build 통과.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1026,9 +1018,9 @@
           <t>8b DB 저장 실측</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1038,7 +1030,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>실제 로그인 상태로 발주를 확정하고 F5 새로고침 후에도 주문이 남아 있는지 사람이 직접 확인합니다. 코드는 이미 완성.</t>
+          <t>실제 로그인 상태로 발주를 여러 건 확정하고 F5 새로고침 후에도 주문이 남아 있는 것을 확인했습니다.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1048,12 +1040,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>실로그인 가능해야 함(이메일 매직링크 rate limit 주의 — 시간 두고 시도).</t>
+          <t>완료 — 매직링크 rate limit은 비밀번호 로그인(a696a36)으로 해결.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>로그인→샘플 설치→발주 확정→F5 후 주문 목록 유지 + Supabase Table Editor에서 ordermoa_orders/order_items row 확인.</t>
+          <t>2026-07-07 실측 성공: 비밀번호 로그인 → 발주 여러 건 확정 → F5 후 주문 목록 유지.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1306,62 +1298,64 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>합산표 개선 팩 — 발주 문장 템플릿·누락 검수·색상</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>다음</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>1차</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>매입처 발주 문장을 "OO상사입니다 / 발주 품목입니다 / 1. 콩나물 3박스" 형식으로 바꾸고, 안 담은 품목 카운터·복사 전 경고·매입처 미지정 뱃지·매입처별 연한 색 구분을 넣습니다. 실사용 피드백(2026-07-07) 반영.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>사장님이 실발주 테스트에서 바로 느낀 불편 3가지(문장 형식, 누락 걱정, 매입처 구분)를 한 번에 해결. 전부 화면 작업이라 DB 변경 없음.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>없음. 설계 확정: docs/order-moa-feedback-design-2026-07-07.md (§2 F1~F4, §6 Codex 프롬프트).</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>개별/전체 복사 문장 형식 테스트, 카운터·경고·뱃지 동작, 인쇄 시 배경색 제거, 모바일 390px. 테스트+빌드 통과.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>docs/order-moa-feedback-design-2026-07-07.md
+web/src/lib/aggregate.ts
+web/src/app/page.tsx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>엑셀/백업/내보내기</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
@@ -1373,72 +1367,119 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>거래처/품목/단가를 엑셀로 한 번에 올리고, 내 데이터를 엑셀/파일로 내려받아 보관합니다. 샘플 초기화 버튼도 포함.</t>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>초기 세팅을 빠르게 하고, 공유 DB에 대한 보험(백업)이 됩니다. 1차 흐름 완성이 먼저라 보류.</t>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>기준정보 CRUD(W02~W04) 완성.</t>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>엑셀 업로드 미리보기→확인→반영, 실패 행 리포트. 내보내기 파일 열림 확인.</t>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>docs/order-moa-expanded-roadmap.md(1.5차)</t>
+          <t>docs/delivery-note-print-spec.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>엑셀/백업/내보내기</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>거래처/품목/단가를 엑셀로 한 번에 올리고, 내 데이터를 엑셀/파일로 내려받아 보관합니다. 샘플 초기화 버튼도 포함.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>초기 세팅을 빠르게 하고, 공유 DB에 대한 보험(백업)이 됩니다. 1차 흐름 완성이 먼저라 보류.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>기준정보 CRUD(W02~W04) 완성.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>엑셀 업로드 미리보기→확인→반영, 실패 행 리포트. 내보내기 파일 열림 확인.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>docs/order-moa-expanded-roadmap.md(1.5차)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>
@@ -1513,12 +1554,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>주문 DB 저장 코드 (8b)</t>
+          <t>주문 DB 저장 실측 (8b/W08)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>확정한 주문이 DB에 저장되는 코드 완성. 실사용 확인(W08)만 남음</t>
+          <t>확정한 주문이 DB에 저장되고, 새로고침 후 주문 목록에 남는 것을 실제 로그인 상태에서 확인 완료</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: improve supplier purchase checklist flow
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W05/W06/W08 실측 완료(0004 적용 + 비밀번호 로그인 + 주문 저장 F5 유지). 다음: W17 합산표 개선 팩(발주 문장 템플릿·누락 검수·색상) → W07 매입처 관리 → W03 품목·별칭.</t>
+          <t>W17 합산표 개선 팩 완료(발주 문장 템플릿·누락 검수 카운터/경고·미지정 뱃지·매입처 파스텔 색·F1 문구, 브라우저 실측). 다음: W07 매입처 관리 → W03 품목·별칭.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 5 · 다음 9 · 보류 3</t>
+          <t>총 17개 — 완료 6 · 다음 8 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -1306,9 +1306,9 @@
           <t>합산표 개선 팩 — 발주 문장 템플릿·누락 검수·색상</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: add supplier management screen
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W17 합산표 개선 팩 완료(발주 문장 템플릿·누락 검수 카운터/경고·미지정 뱃지·매입처 파스텔 색·F1 문구, 브라우저 실측). 다음: W07 매입처 관리 → W03 품목·별칭.</t>
+          <t>W07 매입처 관리 완료(supplier-store + 화면, 추가/수정/보관/복원, 데모 실측·DB 모드는 코드 검증). W17 완료. 다음: W03 품목·별칭 관리(품목 폼에 매입처 드롭다운 포함).</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 6 · 다음 8 · 보류 3</t>
+          <t>총 17개 — 완료 7 · 다음 7 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -970,9 +970,9 @@
           <t>매입처 관리 화면</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: add product alias management
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W07 매입처 관리 완료(supplier-store + 화면, 추가/수정/보관/복원, 데모 실측·DB 모드는 코드 검증). W17 완료. 다음: W03 품목·별칭 관리(품목 폼에 매입처 드롭다운 포함).</t>
+          <t>W03 품목·별칭 관리 완료(product-store + 화면: 품목 CRUD·보관/복원·별칭 칩·기본 매입처 드롭다운, 데모 실측·DB는 코드 검증). W17·W07도 완료. 다음: W04 단가 관리 또는 W09~W11(8c).</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 7 · 다음 7 · 보류 3</t>
+          <t>총 17개 — 완료 8 · 다음 6 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -774,9 +774,9 @@
           <t>기준정보 CRUD — 품목/별칭 관리</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: add price management and supplier contact fields
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W03 품목·별칭 관리 완료(product-store + 화면: 품목 CRUD·보관/복원·별칭 칩·기본 매입처 드롭다운, 데모 실측·DB는 코드 검증). W17·W07도 완료. 다음: W04 단가 관리 또는 W09~W11(8c).</t>
+          <t>W04 단가 관리 완료 + W07 확장(매입처 연락처/주소, 0005 마이그레이션 — [적용 필요] docs/guide-apply-0005-supplier-contact.md). 기준정보 4종(거래처/매입처/품목·별칭/단가) 완성. 다음: W09~W11(8c).</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 8 · 다음 6 · 보류 3</t>
+          <t>총 17개 — 완료 9 · 다음 5 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -823,9 +823,9 @@
           <t>기준정보 CRUD — 단가 관리</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>매입처 이름을 추가·수정·보관하고, 품목별 기본 매입처를 바꾸는 화면(기준정보의 4번째 탭).</t>
+          <t>매입처 이름을 추가·수정·보관하고, 품목별 기본 매입처를 바꾸는 화면(기준정보의 4번째 탭). 2026-07-07 확장: 거래처처럼 연락처·주소 기본정보 추가(0005 마이그레이션 — Supabase 적용 필요).</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: add order raw text retention controls
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W04 단가 관리 완료 + W07 확장(매입처 연락처/주소, 0005 마이그레이션 — [적용 필요] docs/guide-apply-0005-supplier-contact.md). 기준정보 4종(거래처/매입처/품목·별칭/단가) 완성. 다음: W09~W11(8c).</t>
+          <t>W09 발주 원문 저장/삭제 구현·데모 실측 완료 — DB 모드는 0006 마이그레이션 [적용 필요] docs/guide-apply-0006-order-import-link.md. 기준정보 4종 + W09까지 완료. 다음: W10(저장 주문 기반 합산표) → W11(명세서 재출력).</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 9 · 다음 5 · 보류 3</t>
+          <t>총 17개 — 완료 10 · 다음 4 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -584,11 +584,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>a696a36 feat: add password login fallback
-38f4e6c fix: harden supplier migration guidance
-7d3de93 feat: add customer management and supplier persistence
-34d30df docs: refine ordermoa roadmap progress board
-fc59baa docs: add ordermoa system planning charter</t>
+          <t>6ff34f7 docs: record db mode validation
+bdc1323 docs: update next session handoff after final review
+89315d2 feat: add price management and supplier contact fields
+2acb14f feat: add product alias management
+d36cfae feat: add supplier management screen</t>
         </is>
       </c>
     </row>
@@ -1066,9 +1066,9 @@
           <t>8c — 발주 원문(raw_text) 저장/삭제</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1078,28 +1078,30 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>붙여넣은 카톡 원문을 DB에 보관하고, 원하면 삭제할 수 있게 합니다. 삭제해도 확정 주문은 그대로 남습니다.</t>
+          <t>붙여넣은 카톡 원문을 주문에 함께 보관하고, 주문 상세(명세서 화면)에서 원문 보기/삭제를 할 수 있게 했습니다. 삭제해도 주문·금액·명세서는 그대로 남습니다. 코드·데모 실측 완료. DB 모드는 0006 마이그레이션 적용 후 동작(guide-apply-0006-order-import-link.md).</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>"내가 뭐라고 보냈는데?" 분쟁이나 파싱 실수 확인 때 원문이 근거가 됩니다. 테이블은 이미 있는데 앱이 안 쓰고 있음.</t>
+          <t>"내가 뭐라고 보냈는데?" 분쟁이나 파싱 실수 확인 때 원문이 근거가 됩니다. 원문은 개인정보일 수 있어 삭제 가능해야 합니다.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>W08(저장 실측) 통과.</t>
+          <t>W08(저장 실측) 통과. order_imports에 order_id 링크가 없어 0006 마이그레이션 제안(Codex 승인·Supabase 적용 필요).</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>발주 확정→order_imports에 원문 row 확인→원문 삭제→주문은 유지되고 원문만 비워짐.</t>
+          <t>데모: 발주 확정→주문 상세에서 원문 보기→삭제→주문/금액/명세서 유지 확인 완료(2026-07-08). DB: 0006 적용 후 로그인 상태에서 F5 유지 실측 필요.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>web/supabase/migrations/0001_schema.sql(order_imports)
-docs/function-specification.md(F7, Q1)</t>
+          <t>web/src/lib/order-store.ts
+web/src/app/page.tsx
+web/supabase/migrations/0006_order_import_link.sql
+docs/guide-apply-0006-order-import-link.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record raw text db validation
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W09 발주 원문 저장/삭제 구현·데모 실측 완료 — DB 모드는 0006 마이그레이션 [적용 필요] docs/guide-apply-0006-order-import-link.md. 기준정보 4종 + W09까지 완료. 다음: W10(저장 주문 기반 합산표) → W11(명세서 재출력).</t>
+          <t>W09 발주 원문 저장/삭제 구현·DB 실측 완료 — 0006 마이그레이션 Supabase 적용 완료. 기준정보 4종 + W09까지 완료. 다음: W10(저장 주문 기반 합산표) → W11(명세서 재출력).</t>
         </is>
       </c>
     </row>
@@ -584,11 +584,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>6ff34f7 docs: record db mode validation
+          <t>ed2898c feat: add order raw text retention controls
+6ff34f7 docs: record db mode validation
 bdc1323 docs: update next session handoff after final review
 89315d2 feat: add price management and supplier contact fields
-2acb14f feat: add product alias management
-d36cfae feat: add supplier management screen</t>
+2acb14f feat: add product alias management</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>붙여넣은 카톡 원문을 주문에 함께 보관하고, 주문 상세(명세서 화면)에서 원문 보기/삭제를 할 수 있게 했습니다. 삭제해도 주문·금액·명세서는 그대로 남습니다. 코드·데모 실측 완료. DB 모드는 0006 마이그레이션 적용 후 동작(guide-apply-0006-order-import-link.md).</t>
+          <t>붙여넣은 카톡 원문을 주문에 함께 보관하고, 주문 상세(명세서 화면)에서 원문 보기/삭제를 할 수 있게 했습니다. 삭제해도 주문·금액·명세서는 그대로 남습니다. 0006 마이그레이션 적용 후 DB 모드 실측까지 완료했습니다.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1088,12 +1088,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>W08(저장 실측) 통과. order_imports에 order_id 링크가 없어 0006 마이그레이션 제안(Codex 승인·Supabase 적용 필요).</t>
+          <t>완료 — W08(저장 실측) 통과, 0006_order_import_link.sql Supabase 적용 완료.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>데모: 발주 확정→주문 상세에서 원문 보기→삭제→주문/금액/명세서 유지 확인 완료(2026-07-08). DB: 0006 적용 후 로그인 상태에서 F5 유지 실측 필요.</t>
+          <t>2026-07-08 DB 실측: 로그인 상태에서 발주 확정→주문 상세 원문 보기→원문 삭제→F5 후 삭제 상태 유지, 주문/금액/명세서 유지 확인.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1612,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1662,12 +1662,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>파서/합산/검색/주문 저장 빌더/거래처·매입처 보강 자동 테스트</t>
+          <t>파서/합산/검색/주문 저장 빌더/거래처·매입처·raw_text 자동 테스트</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>통과 83/83</t>
+          <t>통과 102/102</t>
         </is>
       </c>
     </row>
@@ -1725,32 +1725,49 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>8a RLS 검증</t>
+          <t>Supabase SQL 0004/0005/0006</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>회사 row, anon 차단, policy, A/B 격리, 위조 insert 차단</t>
+          <t>매입처·연락처·발주 원문 주문 연결</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>통과</t>
+          <t>적용 성공</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>8a RLS 검증</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>회사 row, anon 차단, policy, A/B 격리, 위조 insert 차단</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>민감정보</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>service role key 커밋/번들 포함 여부</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>미포함</t>
         </is>

</xml_diff>

<commit_message>
feat: clarify saved-order aggregate flow
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W09 발주 원문 저장/삭제 구현·DB 실측 완료 — 0006 마이그레이션 Supabase 적용 완료. 기준정보 4종 + W09까지 완료. 다음: W10(저장 주문 기반 합산표) → W11(명세서 재출력).</t>
+          <t>W10 저장 주문 기반 합산표 완료(기존 aggregate·loadOrders 재사용, 마이그레이션 없음) + 대시보드 문구 정합성 보정. 기준정보 4종·W09·W10 완료. 다음: W11(저장 주문 기반 거래명세서 재출력).</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 10 · 다음 4 · 보류 3</t>
+          <t>총 17개 — 완료 11 · 다음 3 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -584,11 +584,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ed2898c feat: add order raw text retention controls
+          <t>755188c docs: record raw text db validation
+ed2898c feat: add order raw text retention controls
 6ff34f7 docs: record db mode validation
 bdc1323 docs: update next session handoff after final review
-89315d2 feat: add price management and supplier contact fields
-2acb14f feat: add product alias management</t>
+89315d2 feat: add price management and supplier contact fields</t>
         </is>
       </c>
     </row>
@@ -1116,9 +1116,9 @@
           <t>8c — 저장 주문 기반 합산표</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>오늘 것뿐 아니라 과거 저장된 주문에서도 날짜/거래처를 골라 합산표를 다시 뽑을 수 있게 합니다.</t>
+          <t>DB에 저장된 주문(loadOrders)을 기준으로 날짜·거래처를 골라 합산표를 다시 뽑습니다. 새로고침·재접속해도 같은 표가 나옵니다. 기존 aggregate 계산 함수 재사용 — 새 마이그레이션 없음. 합산표가 저장 주문 기반 재조회임을 알리는 문구/주문 건수/빈 조건 안내·필터 초기화를 보강.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1138,18 +1138,19 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>W08 통과. (합산 계산 함수는 이미 완성 — DB 조회 결과를 넣기만 하면 됨)</t>
+          <t>완료 — W08(저장 실측). 합산 계산 함수 기존 것, orders 상태가 DB 모드에서 loadOrders 결과라 별도 재조회 로직 불필요.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>주문 저장→앱 재시작→날짜 필터로 같은 합산표 재현.</t>
+          <t>데모 실측(2026-07-08): 날짜/거래처 필터로 주문 건수·품목 합산 확인, 빈 조건 안내+필터 초기화 동작. DB: orders=loadOrders라 F5 시 로드 이펙트가 동일 주문 재조회→같은 표(W08/W09에서 loadOrders F5 유지 실측 완료). 금액은 저장된 order_items 스냅샷만 사용(현재 단가표 재조회 없음).</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/aggregate.ts
-docs/task-prompt-unit-8-supabase-persistence-flow.md(§8)</t>
+web/src/lib/order-store.ts
+web/src/app/page.tsx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: polish delivery note print layout
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W10 저장 주문 기반 합산표 완료(기존 aggregate·loadOrders 재사용, 마이그레이션 없음) + 대시보드 문구 정합성 보정. 기준정보 4종·W09·W10 완료. 다음: W11(저장 주문 기반 거래명세서 재출력).</t>
+          <t>W11 거래명세서 재출력 + 인쇄 양식 하단 마감 보정 완료(border-collapse·합계 tfoot·비고/인수확인·고정 15행, 데모 실측). 기준정보 4종·W09·W10·W11 완료 → 8c 대부분 마무리. 다음: W12(거래처별 월 합계) 또는 잔여 보강.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 11 · 다음 3 · 보류 3</t>
+          <t>총 17개 — 완료 12 · 다음 2 · 보류 3</t>
         </is>
       </c>
     </row>
@@ -584,11 +584,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>755188c docs: record raw text db validation
+          <t>7d05b6f feat: clarify saved-order aggregate flow
+755188c docs: record raw text db validation
 ed2898c feat: add order raw text retention controls
 6ff34f7 docs: record db mode validation
-bdc1323 docs: update next session handoff after final review
-89315d2 feat: add price management and supplier contact fields</t>
+bdc1323 docs: update next session handoff after final review</t>
         </is>
       </c>
     </row>
@@ -1162,12 +1162,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>8c — 거래명세서 재출력</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+          <t>8c — 거래명세서 재출력 + 인쇄 양식 하단 마감</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1177,28 +1177,30 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>과거 주문의 거래명세서를 언제든 다시 열어 인쇄합니다. 금액은 확정 당시 단가 그대로(지금 단가가 바뀌어도 과거 명세서는 안 변함).</t>
+          <t>저장된 주문(주문 목록→보기)의 거래명세서를 다시 열어 인쇄합니다. 금액은 확정 당시 단가 그대로(order_items 스냅샷, customer_prices 재조회 없음). 인쇄 양식 하단 마감을 보정: 표 선 이어붙임(border-collapse), 공급가 합계를 표 tfoot에 붙여 정렬, 비고/인수확인 마감행, 고정 15행으로 A4 1장 균일 출력. '확정 당시 단가 기준' 안내는 no-print.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>거래처가 "지난주 명세서 다시 주세요" 할 때 필요합니다. 확정 시점 금액 보존은 헌장의 불변 규칙.</t>
+          <t>거래처가 "지난주 명세서 다시 주세요" 할 때 필요합니다. 확정 시점 금액 보존은 헌장의 불변 규칙. 실제 출력물처럼 하단이 깔끔해야 씀.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>W08 통과.</t>
+          <t>완료 — W08(저장). 거래명세서 화면은 이미 존재(주문 목록→보기).</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>주문 저장→단가 변경→과거 명세서 재출력 시 금액이 그대로인지 확인.</t>
+          <t>데모 실측(2026-07-08): 6품목 명세서에서 표 선 연결·합계 tfoot 정렬(76,000)·비고/인수확인 마감·15행 채움 확인, 콘솔 0. 금액은 order.total(저장 스냅샷). DB 재출력 F5는 loadOrders 경로(W08/W09 검증분).</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md
-docs/order-moa-system-meta-prompt.md(§3)</t>
+          <t>web/src/lib/delivery-note.ts
+web/src/app/page.tsx
+web/src/app/globals.css
+docs/delivery-note-print-spec.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add monthly summary and CSV exports
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,11 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -94,6 +99,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -536,7 +544,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W11 거래명세서 재출력 + 인쇄 양식 하단 마감 보정 완료(border-collapse·합계 tfoot·비고/인수확인·고정 15행, 데모 실측). 기준정보 4종·W09·W10·W11 완료 → 8c 대부분 마무리. 다음: W12(거래처별 월 합계) 또는 잔여 보강.</t>
+          <t>W15 데이터 내보내기(CSV) 절반 완료 — '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 CSV, 월 합계 화면에서 월합계 CSV 백업(공유 Supabase 쿼터 대비 안전망). 마이그레이션 없음, 데모 실측. W12 거래처별 월 합계 완료. 다음: 엑셀 가져오기(후순위) 또는 전용 Supabase 분리 논의.</t>
         </is>
       </c>
     </row>
@@ -560,7 +568,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 12 · 다음 2 · 보류 3</t>
+          <t>총 17개 — 완료 13 · 다음 1 · 보류 2 · 진행 중 1</t>
         </is>
       </c>
     </row>
@@ -1215,9 +1223,9 @@
           <t>8c — 거래처별 월 합계</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>다음</t>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1227,27 +1235,29 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>거래처별로 이번 달 얼마 팔았는지 합계를 보여줍니다.</t>
+          <t>조회 메뉴 '거래처별 월 합계'에서 월(YYYY-MM)을 골라 거래처별 주문 건수·공급가 합계·마지막 주문일과 전체 합계를 봅니다. 저장된 확정 주문의 금액(order.total 스냅샷)만 씁니다 — 세금계산서 발행이 아니라 월말 확인용. 순수 함수 monthly-summary.ts + 새 뷰, 마이그레이션 없음.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>월말 정산·세금계산서 발행 금액의 근거 숫자. 별도 계산 없이 저장된 주문에서 바로 나옵니다.</t>
+          <t>월말 '거래처별 이번 달 얼마 팔았나' 확인용 근거 숫자. 별도 계산 없이 저장된 주문에서 바로 나옵니다.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>W08 통과.</t>
+          <t>완료 — W08(저장). loadOrders가 전체 확정 주문을 주므로 그 order.total을 월·거래처로 집계.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>주문 여러 건 저장→거래처×월 합계가 라인 금액 합과 일치.</t>
+          <t>데모 실측(2026-07-08): 2026-07 발주 2건→가람식당 76,000·한빛카페 49,400·전체 125,400 확인. 단가표 콩나물 99,999원 변경 후에도 월 합계 불변(스냅샷). 빈 월 안내. 정렬 금액 내림차순. 콘솔 0.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>docs/task-prompt-unit-8-supabase-persistence-flow.md(§6)
+          <t>web/src/lib/monthly-summary.ts
+web/src/app/monthly-summary-view.tsx
+web/src/app/page.tsx
 docs/function-specification.md(F12, §5.2)</t>
         </is>
       </c>
@@ -1407,39 +1417,42 @@
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>보류</t>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>1차</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>거래처/품목/단가를 엑셀로 한 번에 올리고, 내 데이터를 엑셀/파일로 내려받아 보관합니다. 샘플 초기화 버튼도 포함.</t>
+          <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>초기 세팅을 빠르게 하고, 공유 DB에 대한 보험(백업)이 됩니다. 1차 흐름 완성이 먼저라 보류.</t>
+          <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>기준정보 CRUD(W02~W04) 완성.</t>
+          <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>엑셀 업로드 미리보기→확인→반영, 실패 행 리포트. 내보내기 파일 열림 확인.</t>
+          <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>docs/order-moa-expanded-roadmap.md(1.5차)</t>
+          <t>web/src/lib/csv-export.ts
+web/src/app/page.tsx
+web/src/app/monthly-summary-view.tsx
+docs/task-prompt-W15-export.md</t>
         </is>
       </c>
     </row>
@@ -1665,12 +1678,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>파서/합산/검색/주문 저장 빌더/거래처·매입처·raw_text 자동 테스트</t>
+          <t>파서/합산/검색/주문 저장 빌더/거래처·매입처·raw_text·월합계·CSV 자동 테스트</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>통과 102/102</t>
+          <t>통과 111/111</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: improve order entry date and price workflow
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W15 데이터 내보내기(CSV) 절반 완료 — '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 CSV, 월 합계 화면에서 월합계 CSV 백업(공유 Supabase 쿼터 대비 안전망). 마이그레이션 없음, 데모 실측. W12 거래처별 월 합계 완료. 다음: 엑셀 가져오기(후순위) 또는 전용 Supabase 분리 논의.</t>
+          <t>W18 Phase 1 UX 개선 완료 — 주문일 표시/수정(KST 기준), 파싱 화면 단가 Enter이동+변경단가 전체저장, 주문 목록 날짜 조회(기본 오늘/전체보기). 마이그레이션 없음, 데모 실측(합산표·월합계 무영향 확인). 다음 Phase 2/3(카테고리·다단위·product_units)는 스키마 필요라 분리. 잔여: 엑셀 가져오기, 전용 Supabase 분리 논의.</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 17개 — 완료 13 · 다음 1 · 보류 2 · 진행 중 1</t>
+          <t>총 18개 — 완료 14 · 다음 1 · 보류 2 · 진행 중 1</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1362,92 +1362,141 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>Phase 1 UX 개선 — 주문일·단가 일괄저장·주문목록 날짜조회</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>1차</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>①주문일 표시/수정: 파싱 확인 화면에 주문일 입력칸 추가, 어제 발주도 날짜 바꿔 확정. 날짜는 한국시간(KST) 기준(UTC라 새벽에 전날 저장되던 것 수정). ②파싱 화면 단가 일괄저장: 단가 칸에서 Enter로 다음 칸 이동, 바뀐 단가를 '변경 단가 전체 저장' 한 번으로 저장. ③주문 목록 날짜 조회: 기본 오늘, 날짜 선택·전체 보기. 마이그레이션 없음.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>실사용 불편 3가지 — 어제 발주 날짜 못 바꿈, 단가 한 줄씩 저장 번거로움, 주문 목록이 전부 섞여 보임. 합산표·월합계는 전역 orders 그대로 써서 안 깨지게.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>W08~W12(저장 주문 흐름).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>데모 실측(2026-07-08): KST 주문일·어제로 확정→목록 해당 날짜, 단가 2개 변경→Enter 이동→일괄저장(2)→재파싱 자동적용, 목록 오늘/전체/빈상태, 합산표·월합계 무영향. 순수함수 테스트(todayKst 3·collectPriceChanges 3). root5·web117·build·audit0.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>web/src/lib/date-utils.ts
+web/src/lib/price-store.ts
+web/src/app/page.tsx</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1456,48 +1505,48 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>
@@ -1678,12 +1727,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>파서/합산/검색/주문 저장 빌더/거래처·매입처·raw_text·월합계·CSV 자동 테스트</t>
+          <t>파서/합산/검색/주문 저장 빌더/거래처·매입처·raw_text·월합계·CSV·KST 날짜·단가 일괄 저장 자동 테스트</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>통과 111/111</t>
+          <t>통과 117/117</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: harden parser for field order text
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,17 +58,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -99,9 +94,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -544,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W18 Phase 1 UX 개선 완료 — 주문일 표시/수정(KST 기준), 파싱 화면 단가 Enter이동+변경단가 전체저장, 주문 목록 날짜 조회(기본 오늘/전체보기). 마이그레이션 없음, 데모 실측(합산표·월합계 무영향 확인). 다음 Phase 2/3(카테고리·다단위·product_units)는 스키마 필요라 분리. 잔여: 엑셀 가져오기, 전용 Supabase 분리 논의.</t>
+          <t>W13 실제 발주 테스트 1차 라운드 완료 — 현장식 문장(공백 다품목·붙여쓰기·종결어미·조사·규격숫자)으로 파서 검증. order-parser.ts 최소 보강 2건: (1) 한 줄에 수량단위 클러스터 2개↑면 라인 분리(뒤 품목 조용히 유실되던 치명 문제 해결, 규격+수량은 분리 안 함), (2) 종결어미 이요·조사 는/은 제거. real-order-fixture.test.ts에 W13 섹션 11건 추가 → web 117→128. 마이그레이션·스키마 0, 스냅샷 원칙 유지. 다음: Phase 2(카테고리)·엑셀 가져오기·전용 Supabase 분리.</t>
         </is>
       </c>
     </row>
@@ -568,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 18개 — 완료 14 · 다음 1 · 보류 2 · 진행 중 1</t>
+          <t>총 18개 — 완료 14 · 진행 중 2 · 보류 2</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1267,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>다음</t>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1285,7 +1277,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>실제 받았던 발주(가명 처리)를 길게 여러 번 넣어보며 파싱·검색·매입처 분리가 현장에서 통하는지 반복 확인합니다.</t>
+          <t>실제 받았던 발주(가명 처리)를 길게 여러 번 넣어보며 파싱·검색·매입처 분리가 현장에서 통하는지 반복 확인합니다. 1차 라운드(2026-07-08) 완료: 현장식 문장으로 파서 보강 2건.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1300,7 +1292,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>장문 발주 10건 이상 투입→미매칭/오인식을 fixture 테스트로 남기고 파서 보강.</t>
+          <t>1차(2026-07-08): 현장식 문장 검증→파서 보강 2건(한 줄 공백/붙여쓰기 다품목 분리·뒤 품목 유실 방지, 종결어미 이요·조사 는/은 제거) + fixture 11건(web 128). 브라우저 데모 smoke 2건(확정→명세서→합산표). 실제 수령 발주 확보 시 라운드 반복.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1466,7 +1458,7 @@
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>

</xml_diff>

<commit_message>
feat: add product categories
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W13 실제 발주 테스트 1차 라운드 완료 — 현장식 문장(공백 다품목·붙여쓰기·종결어미·조사·규격숫자)으로 파서 검증. order-parser.ts 최소 보강 2건: (1) 한 줄에 수량단위 클러스터 2개↑면 라인 분리(뒤 품목 조용히 유실되던 치명 문제 해결, 규격+수량은 분리 안 함), (2) 종결어미 이요·조사 는/은 제거. real-order-fixture.test.ts에 W13 섹션 11건 추가 → web 117→128. 마이그레이션·스키마 0, 스냅샷 원칙 유지. 다음: Phase 2(카테고리)·엑셀 가져오기·전용 Supabase 분리.</t>
+          <t>Phase 2 W19 — 품목 카테고리 6종(농산물/공산품/냉식/육류/수산/기타). 6종 고정이라 별도 테이블 없이 ordermoa_products.category 컬럼 1개(text NOT NULL DEFAULT '기타' CHECK 6종). 마이그레이션 0007 작성 완료, 적용은 Codex 승인 후 SQL Editor(guide-apply-0007-product-category.md). 0007 미적용 DB도 안 깨지게 읽기/쓰기 폴백(isMissingCategoryColumn). 품목·별칭 관리에 카테고리 select·목록·필터. order_items·합산표·명세서·월합계·파서 전부 무변경(스냅샷 무관). 카테고리 상수 단일 소스 product-category.ts. web 128→133, root5·build·audit0. 다음: Phase 3(product_units) 또는 엑셀 가져오기·전용 Supabase 분리.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 18개 — 완료 14 · 진행 중 2 · 보류 2</t>
+          <t>총 19개 — 완료 14 · 진행 중 3 · 보류 2</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1403,92 +1403,142 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>Phase 2 — 품목 카테고리 6종</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>품목을 6종(농산물/공산품/냉식/육류/수산/기타)으로 분류합니다. 품목·별칭 관리 화면에서 카테고리를 고르고, 목록을 카테고리로 걸러 봅니다. DB에는 컬럼 하나(category)만 추가 — 6종 고정이라 별도 표는 안 만듭니다. 코드는 완료, DB 반영(0007)은 Codex 승인 후 적용 대기.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>품목이 늘면 종류별로 묶어 봐야 관리·발주가 편합니다. 사장님 실사용 피드백. 스키마가 필요해 별도 세션으로 분리했고, 컬럼 1개라 위험 낮음.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>W03(품목 관리). 0007 적용은 Codex 승인 게이트.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>코드 완료(2026-07-09): 데모 smoke — 목록 카테고리 표시·필터(냉식 5종)·신규 육류 품목 추가·회귀(발주→확정→합산표) 정상, 콘솔 앱오류 0. TDD web 128→133. 0007 미적용 DB 폴백(안 깨짐). 적용 후 DB 실측은 guide-apply-0007 가이드 체크리스트. 스냅샷·집계 무변경.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>web/src/lib/product-category.ts
+web/src/lib/product-store.ts
+web/supabase/migrations/0007_product_category.sql
+docs/guide-apply-0007-product-category.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1497,48 +1547,48 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>

<commit_message>
chore: add real catalog extraction draft
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Phase 2 W19 — 품목 카테고리 6종(농산물/공산품/냉식/육류/수산/기타). 6종 고정이라 별도 테이블 없이 ordermoa_products.category 컬럼 1개(text NOT NULL DEFAULT '기타' CHECK 6종). 마이그레이션 0007 작성 완료, 적용은 Codex 승인 후 SQL Editor(guide-apply-0007-product-category.md). 0007 미적용 DB도 안 깨지게 읽기/쓰기 폴백(isMissingCategoryColumn). 품목·별칭 관리에 카테고리 select·목록·필터. order_items·합산표·명세서·월합계·파서 전부 무변경(스냅샷 무관). 카테고리 상수 단일 소스 product-category.ts. web 128→133, root5·build·audit0. 다음: Phase 3(product_units) 또는 엑셀 가져오기·전용 Supabase 분리.</t>
+          <t>W20 — 실제 엑셀 기반 품목 기준정보 초안. 친구 실운영 이카운트 엑셀(품목마스터+단가마스터, 저장소 밖·미커밋)을 품목코드로 조인→정제해 docs/order-moa-catalog-real-draft.json(1590품목, 588KB) 산출. scripts/extract-real-catalog.py(경로 인자·self-check). 괄호 화이트리스트로 공급사/브랜드 제거→식별정보 자체 스캔 0건, 단가 100원 반올림, 카테고리 6종 키워드 초안(자동 60.8%·나머지 needsReview). import(DB 반영)는 W21로 분리 — 이번은 검수 초안까지만. .gitignore에 원시데이터 유출 안전망 추가. 앱 코드 무변경(web 133 그대로). 사용자 결정: 상호 제외·품목/단위/단가는 실 엑셀 우선. 관찰: 다규격/다단위 210그룹(Phase3 근거), 6종이 조미료/가공 못 담음. 다음: W21 import 미리보기/검수+DB반영(Codex 승인), 0007 적용, 전용 Supabase 분리.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 19개 — 완료 14 · 진행 중 3 · 보류 2</t>
+          <t>총 20개 — 완료 14 · 진행 중 4 · 보류 2</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1453,92 +1453,141 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>실제 엑셀 기반 품목 기준정보 초안</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>친구가 실제로 운영하며 내려받은 이카운트 엑셀(품목마스터+단가마스터)에서 품목명·규격·단위·단가 패턴을 뽑아 검수용 초안(catalog-real-draft.json, 1590품목)을 만들었습니다. 가명/더미 샘플 33종 대신 실제 현장 품목 패턴을 기준으로 삼기 위함. 상호·거래처·공급처 등 식별정보는 아예 안 읽고 제외했고, 단가는 100원 반올림. import(DB 반영)는 W21에서.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>실 베타는 품목 수가 많아 샘플 33종으론 부족. 사용자 결정: 상호는 제외하되 품목·단위·단가는 실제 엑셀 패턴 우선. import 전에 검수 가능한 산출물이 있어야 안전.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>원본 엑셀은 저장소 밖. 추출 스크립트만 커밋. import/DB 반영은 W21(Codex 승인).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>scripts/extract-real-catalog.py(self-check 6종) → 초안 JSON 1590품목. 식별정보 자체 스캔 0건(괄호 화이트리스트로 공급사/브랜드 제거). 카테고리 자동 60.8%(나머지 needsReview). 관찰: 다규격/다단위 210그룹=Phase3 근거, 조미료/가공은 6종 밖(기타). 앱 코드 무변경 → web 133 그대로.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>scripts/extract-real-catalog.py
+docs/order-moa-catalog-real-draft.json
+docs/agent-worklog.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1547,48 +1596,48 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>

<commit_message>
feat: add catalog import workflow
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W20 — 실제 엑셀 기반 품목 기준정보 초안. 친구 실운영 이카운트 엑셀(품목마스터+단가마스터, 저장소 밖·미커밋)을 품목코드로 조인→정제해 docs/order-moa-catalog-real-draft.json(1590품목, 588KB) 산출. scripts/extract-real-catalog.py(경로 인자·self-check). 괄호 화이트리스트로 공급사/브랜드 제거→식별정보 자체 스캔 0건, 단가 100원 반올림, 카테고리 6종 키워드 초안(자동 60.8%·나머지 needsReview). import(DB 반영)는 W21로 분리 — 이번은 검수 초안까지만. .gitignore에 원시데이터 유출 안전망 추가. 앱 코드 무변경(web 133 그대로). 사용자 결정: 상호 제외·품목/단위/단가는 실 엑셀 우선. 관찰: 다규격/다단위 210그룹(Phase3 근거), 6종이 조미료/가공 못 담음. 다음: W21 import 미리보기/검수+DB반영(Codex 승인), 0007 적용, 전용 Supabase 분리.</t>
+          <t>W21 — 카탈로그 import 미리보기/검수 + 선택 DB 반영. W20 초안(1590품목) JSON을 데이터 화면에서 업로드→요약/필터/50페이지/행편집/중복명 경고/기존일치 검수→선택분만 반영. DB 모드는 0007(category)+0008(source_code) 적용 후 200건 배치 insert/update, source_code 멱등 재분류, 별칭 충돌 무시 upsert, 반영 후 products 재조회. 데모 모드는 메모리 반영. 매핑: 입고단가→base_purchase_price, 출고단가는 저장 안 함(기본 판매단가는 Phase 3), category→products.category, code→source_code. order_items·집계·파서 무변경(스냅샷 유지). 다음: 로그인 모드 10~20건 소량 DB smoke, 전용 Supabase 분리 vs Phase 3.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 20개 — 완료 14 · 진행 중 4 · 보류 2</t>
+          <t>총 21개 — 완료 16 · 진행 중 3 · 보류 2</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1265,9 +1265,9 @@
           <t>실제 발주 테스트 라운드</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>품목을 6종(농산물/공산품/냉식/육류/수산/기타)으로 분류합니다. 품목·별칭 관리 화면에서 카테고리를 고르고, 목록을 카테고리로 걸러 봅니다. DB에는 컬럼 하나(category)만 추가 — 6종 고정이라 별도 표는 안 만듭니다. 코드는 완료, DB 반영(0007)은 Codex 승인 후 적용 대기.</t>
+          <t>품목을 6종(농산물/공산품/냉식/육류/수산/기타)으로 분류합니다. 품목·별칭 관리 화면에서 카테고리를 고르고, 목록을 카테고리로 걸러 봅니다. DB에는 컬럼 하나(category)만 추가 — 6종 고정이라 별도 표는 안 만듭니다. 코드 완료, 0007 Supabase 적용 완료.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1461,9 +1461,9 @@
           <t>실제 엑셀 기반 품목 기준정보 초안</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1502,92 +1502,142 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>카탈로그 import (미리보기/검수 + 반영)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>W20 초안(JSON)을 앱에서 올려 미리보기로 검수하고, 고른 품목만 기준정보로 반영하는 화면입니다. 업로드·요약·필터·행편집·중복명 경고·기존일치 표시를 제공하고, 데모는 화면 반영, 로그인 DB 모드는 200건 배치 insert/update와 source_code 멱등 매칭으로 영구 반영합니다. 출고단가는 참고만 하고 저장 안 함(기본 판매단가는 이후).</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>샘플 33종으론 부족한 현장 품목을, 검수를 거쳐 안전하게 기준정보로 올리기 위함. 잘못된 대량 반영·중복 품목을 막는 게 핵심.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>W20 초안. 0007(카테고리)+0008(source_code) SQL Editor 적용 완료(사용자 확인). 공유 Supabase 쿼터 부담 때문에 전체 반영 전 소량 smoke 권장.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>2026-07-09: catalog-import.ts/test + catalog-import-view.tsx. 데모 smoke — 업로드 8건→기존일치/중복명/검토 뱃지, 중복명 동시선택 경고+차단, 신규 4건 반영→품목관리·파서 매칭, 앱오류 0. W21-B: applyCatalogImportToDb 추가(source_code 멱등 재분류, 200건 배치, 별칭 upsert, 반영 후 reload). 로그인 DB 소량 실측은 다음 확인 포인트.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>web/src/lib/catalog-import.ts
+web/src/app/catalog-import-view.tsx
+web/supabase/migrations/0008_product_source_code.sql
+docs/guide-apply-0008-product-source-code.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1596,48 +1646,48 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>

<commit_message>
feat: add product base sale price
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W21 — 카탈로그 import 미리보기/검수 + 선택 DB 반영. W20 초안(1590품목) JSON을 데이터 화면에서 업로드→요약/필터/50페이지/행편집/중복명 경고/기존일치 검수→선택분만 반영. DB 모드는 0007(category)+0008(source_code) 적용 후 200건 배치 insert/update, source_code 멱등 재분류, 별칭 충돌 무시 upsert, 반영 후 products 재조회. 데모 모드는 메모리 반영. 매핑: 입고단가→base_purchase_price, 출고단가는 저장 안 함(기본 판매단가는 Phase 3), category→products.category, code→source_code. order_items·집계·파서 무변경(스냅샷 유지). 다음: 로그인 모드 10~20건 소량 DB smoke, 전용 Supabase 분리 vs Phase 3.</t>
+          <t>W22 — 품목 기본 출고단가(base_sale_price) 도입. 베타 검증에서 금액이 0원으로만 나오지 않게, 엑셀 출고단가를 products.base_sale_price에 저장하고 파싱 단가 우선순위를 거래처별 단가(customer_prices) &gt; 품목 기본 출고단가 &gt; 미등록으로 변경. customer_prices 자동 생성 없음, order_items.unit_price 스냅샷 불변. 0009 마이그레이션 작성(적용 대기), 카탈로그 재import 시 source_code 멱등으로 기존 품목 base_sale_price 갱신.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 21개 — 완료 16 · 진행 중 3 · 보류 2</t>
+          <t>총 22개 — 완료 16 · 진행 중 4 · 보류 2</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>W20 초안. 0007(카테고리)+0008(source_code) SQL Editor 적용 완료(사용자 확인). 공유 Supabase 쿼터 부담 때문에 전체 반영 전 소량 smoke 권장.</t>
+          <t>W20 초안. 0007(카테고리)+0008(source_code) SQL Editor 적용 완료(사용자 확인). Usage 확인 결과 용량 여유 있음 — 전체 반영 리스크는 쿼터보다 중복명/검토필요 데이터 품질.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09: catalog-import.ts/test + catalog-import-view.tsx. 데모 smoke — 업로드 8건→기존일치/중복명/검토 뱃지, 중복명 동시선택 경고+차단, 신규 4건 반영→품목관리·파서 매칭, 앱오류 0. W21-B: applyCatalogImportToDb 추가(source_code 멱등 재분류, 200건 배치, 별칭 upsert, 반영 후 reload). 로그인 DB 소량 실측은 다음 확인 포인트.</t>
+          <t>2026-07-09: catalog-import.ts/test + catalog-import-view.tsx. 데모 smoke — 업로드 8건→기존일치/중복명/검토 뱃지, 중복명 동시선택 경고+차단, 신규 4건 반영→품목관리·파서 매칭, 앱오류 0. W21-B: applyCatalogImportToDb 추가(source_code 멱등 재분류, 200건 배치, 별칭 upsert, 반영 후 reload). 사용자 DB 소량 실측: 품목 반영/F5 유지/재반영 중복 없음/파싱 매칭 확인.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1552,92 +1552,142 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W22</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>품목 기본 출고단가</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>진행 중</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>엑셀 출고단가를 품목 기본 출고단가(base_sale_price)로 저장하고, 거래처별 단가가 없을 때 발주 파싱 금액 fallback으로 씁니다. 거래처별 단가(customer_prices)가 있으면 항상 우선하고, customer_prices를 자동 생성하지는 않습니다.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>베타 검증에서 품목은 매칭되지만 판매금액이 전부 0원이면 주문/명세서/합산표 검증이 어렵습니다. 다단위(product_units) 전 단계의 최소 구조로 기본 출고단가 자리를 마련합니다.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>W21 카탈로그 import. 0009_product_base_sale_price.sql Supabase 적용 후 같은 카탈로그를 재import하면 source_code 멱등으로 기존 품목의 base_sale_price가 채워짐.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>코드 검증: resolveSalePrice 단가 우선순위(customer &gt; base &gt; none), 파서 fallback, catalog import repSalePrice→base_sale_price, product-store 매핑 테스트. 적용 후 실측: 거래처 단가 없는 품목이 기본 단가 적용으로 금액 표시, 거래처별 단가가 있으면 우선, customer_prices 새 row 없음, 과거 주문 스냅샷 불변.</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>web/src/lib/domain/index.ts
+web/src/lib/order-parser.ts
+web/supabase/migrations/0009_product_base_sale_price.sql
+docs/guide-apply-0009-product-base-sale-price.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1646,48 +1696,48 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>

<commit_message>
docs: redesign dual-path order workflow
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -58,12 +58,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -500,7 +500,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>전체 ERP 대체가 아니라, 도소매/식당납품 사장님용 좁은 웹 ERP MVP. 핵심 가치: 카톡/문자 발주를 붙여넣으면 파싱, 합산표, 매입처별 발주 문장, 거래명세서까지 이어지는 것.</t>
+          <t>전체 ERP 대체가 아니라, 중간 납품업자의 흩어진 발주를 모아 품목·수량을 확인하고 합산·매입처 발주로 이은 뒤, 준비된 판매가격 또는 매입가 확인 후 마감한 가격으로 거래명세서까지 연결하는 반응형 웹 업무 도구.</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W22 — 품목 기본 출고단가(base_sale_price) 도입. 베타 검증에서 금액이 0원으로만 나오지 않게, 엑셀 출고단가를 products.base_sale_price에 저장하고 파싱 단가 우선순위를 거래처별 단가(customer_prices) &gt; 품목 기본 출고단가 &gt; 미등록으로 변경. customer_prices 자동 생성 없음, order_items.unit_price 스냅샷 불변. 0009 마이그레이션 작성(적용 대기), 카탈로그 재import 시 source_code 멱등으로 기존 품목 base_sale_price 갱신.</t>
+          <t>W23-R1 준비 — 선택형 두 경로의 문서 재설계는 완료. 다음은 가격 대기 주문의 상태·저장 모델을 설계하고 기존 확정 주문·unit_price 스냅샷·generated amount·합산표·명세서가 손상되지 않는지 검증하는 승인 게이트입니다. 코드·SQL 작성 전 orders 단일 소스와 별도 초안 객체를 비교하고, 단일 소스 안에서는 기존 draft 재사용 vs 신규 상태, unit_price nullable vs 별도 가격 상태/시각을 비교합니다.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 22개 — 완료 16 · 진행 중 4 · 보류 2</t>
+          <t>총 23개 — 완료 20 · 보류 2 · 진행 중 1</t>
         </is>
       </c>
     </row>
@@ -584,11 +584,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>7d05b6f feat: clarify saved-order aggregate flow
-755188c docs: record raw text db validation
-ed2898c feat: add order raw text retention controls
-6ff34f7 docs: record db mode validation
-bdc1323 docs: update next session handoff after final review</t>
+          <t>f563f50 docs: plan dual confirmation workflow redesign
+c3dc098 fix: exclude base sale price fallback lines from bulk price save
+222920a feat: add product base sale price
+f1a3a58 docs: record catalog import smoke plan
+66d1af2 feat: add catalog import workflow</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1411,9 +1411,9 @@
           <t>Phase 2 — 품목 카테고리 6종</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1510,9 +1510,9 @@
           <t>카탈로그 import (미리보기/검수 + 반영)</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1560,9 +1560,9 @@
           <t>품목 기본 출고단가</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>진행 중</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>W21 카탈로그 import. 0009_product_base_sale_price.sql Supabase 적용 후 같은 카탈로그를 재import하면 source_code 멱등으로 기존 품목의 base_sale_price가 채워짐.</t>
+          <t>완료 — W21 카탈로그 import, 0009_product_base_sale_price.sql Supabase 적용, 같은 카탈로그 재import를 통한 기존 품목 base_sale_price 갱신까지 실측.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1602,92 +1602,142 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W23</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>전체 시스템 재설계 — 두 경로·가격 마감 (문서 개편)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>실사용 인터뷰에서 '단위 생략 카톡 발주는 거래처별 관습 문제'와 '판매단가는 매입처 명세서를 받은 뒤 그때그때 결정'이 확인됐습니다. 그래서 기존 '가격 포함 바로 확정'을 유지한 채, '수량 먼저 확인 → 합산·매입처 발주 → 매입가 입력 → 가격 마감(최종 확정)' 경로를 선택형으로 추가하고, 대시보드를 '오늘 업무' 큐로 바꾸는 재설계를 확정했습니다. 이번 회차는 문서 전수 감사·개편까지만 완료(코드/SQL 무변경).</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>단가 마스터 1,500개를 항상 관리해야 돌아가는 구조는 실사용과 맞지 않음. 한 사용자 습관에 과적합하지 않도록 공통 문제(수량이 가격보다 먼저 확정됨)는 핵심에, 개인 방식은 선택 경로로 격리. 과거 주문 스냅샷 불변 원칙은 '판매단가가 최종 확정되는 시점'으로 재정의해 유지.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>구현은 R1(상태·저장 모델 + 마이그레이션 설계, Codex 승인 게이트)부터 별도 세션. 권장 방향은 orders 단일 소스 유지지만 기존 draft 재사용/신규 상태와 unit_price nullable/별도 가격 상태를 비교하기 전 구현 확정 금지. OCR은 '보류된 입력 어댑터 실험'으로 재분류(게이트 3조건 통과 전 착수 금지).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>문서 산출: 감사(order-moa-document-audit-2026-07-11) + 재설계 기준(order-moa-system-redesign-2026-07-11, 15개 절) + 헌장/제품/요구(F14~F19)/기능(§5.3)/화면(§16)/DB/모듈맵(M17~M20)/로드맵(R0~R8)/검수(§12)/검증(§12) 전수 정렬. 코드 무변경 기준선: root 5/5 · web 150/150 · build 성공 · audit 0 · diff-check clean.</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>docs/order-moa-document-audit-2026-07-11.md
+docs/order-moa-system-redesign-2026-07-11.md
+docs/superpowers/specs/2026-07-11-order-moa-dual-confirmation-workflow-design.md
+docs/agent-worklog.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1696,48 +1746,48 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>

<commit_message>
feat: add price close workflow and operation UX plan
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W23-R3 준비 — 수량 확인(가격 대기) 경로는 구현·smoke 완료. 다음은 '가격 마감' 화면: 매입처 명세서를 보고 품목별 매입가 1회 입력 → 거래처별 판매가 제안(거래처 단가 &gt; 기본 출고단가) 확인·수정 → 최종 확정 스냅샷(items UPDATE→orders confirmed 순). 마진 자동화·자동 저장 금지 원칙 유지.</t>
+          <t>W23-R5a 준비 — 가격 마감(R3) + 검수 보강 완료, 0011 가드 SQL 적용 및 로그인 DB 앱 경로 smoke(가격 마감→최종 확정→거래명세서) 확인. 다음은 마이그레이션 없는 운영 UX 팩: 가격 입력 전체선택/Enter, 단가 관리 적용 단가 표시, 매입처 발주 문장 편집·날짜, 이번 발주만 매입처 변경.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 25개 — 완료 22 · 보류 2 · 진행 중 1</t>
+          <t>총 26개 — 완료 23 · 보류 2 · 진행 중 1</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1749,92 +1749,142 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W23-R3</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>가격 마감 — 매입가 입력→판매가 확정→최종 확정</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>가격 대기 주문의 [가격 마감] 버튼을 누르면, 품목별 오늘 매입가를 한 번 입력하고 라인별 판매단가를 확정하는 화면이 열립니다. 거래처 단가·기본 출고단가·최근 확정가를 참고로 보여주고 예상 마진은 표시만(저장 안 함) 하며, 값을 확정하면 최종 확정(스냅샷)되어 거래명세서를 발행할 수 있습니다. 매입가·판매가의 '기본값에도 저장'은 각각 체크했을 때만 반영됩니다.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>W23 두 경로의 마지막 조각. 가격 대기 주문을 실제로 마감할 수단을 제공하고, 확정 시점 스냅샷을 DB 가드로 잠가 무결성을 지킨다. 자동 마진·자동 저장을 배제해 사장님이 값을 통제한다.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>R1(0010)·R2 완료. 0011 가드 보강 SQL은 사용자 SQL Editor에서 적용 완료. 로그인 DB 앱 경로(수량/가격 대기→가격 마감→최종 확정→거래명세서) smoke 완료. H1~H7b raw-DB 가드 실험은 SQL Editor 임시 테이블 세션 제약으로 보류하며, 가이드는 향후 관리자 검증용으로 유지한다.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>web 173/173(planCloseOrderPrices 11 + planCustomerPriceSaves 4 + closeOrderPrices/saveOrder mock 6) · root 5/5 · build 성공 · audit 0 · tsc 통과 · diff-check clean. 검수 보강 5종: 0011 INSERT 가드(confirmed/cancelled 라인 주입 차단, saveOrder를 qc삽입→confirmed 승격으로 재구성) · closeOrderPrices 영향행 1행 검증 · 기준정보 저장 실패 메시지 분리 · 동일 품목 다줄 거래처단가 조용한 덮어쓰기 금지(제외+경고) · confirmed_at 의미 문서화. 데모 smoke: 같은 품목 2줄 8,000/8,500 라인 id 정확 매핑(41,500)·단가 누락 마감 차단·충돌 경고·덮어쓰기 방지·콘솔 0. 미커밋 — Codex 검수 대기.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>web/supabase/migrations/0011_order_pricing_guard_hardening.sql
+docs/guide-apply-0011-order-pricing-guard.md
+docs/order-moa-w23-r1-state-model-decision.md
+docs/agent-worklog.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1843,48 +1893,48 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>

<commit_message>
feat: improve operational order UX
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W23-R5a 준비 — 가격 마감(R3) + 검수 보강 완료, 0011 가드 SQL 적용 및 로그인 DB 앱 경로 smoke(가격 마감→최종 확정→거래명세서) 확인. 다음은 마이그레이션 없는 운영 UX 팩: 가격 입력 전체선택/Enter, 단가 관리 적용 단가 표시, 매입처 발주 문장 편집·날짜, 이번 발주만 매입처 변경.</t>
+          <t>W23-R5a 운영 UX 팩 구현·검수 완료(마이그레이션 0, web 186/186). 가격 입력 전체선택/Enter·단가 관리 적용 단가 표시·매입처 발주 문장 날짜·편집·이번 발주만 매입처 변경, 거래처·날짜 필터 변경 시 임시 재지정·편집본 초기화까지 됨. 다음 후보: W23-R5b 확정 주문 정정(취소→복사→재확정) / W23-R4 대시보드 오늘 업무 큐 / W24 품목코드·과세구분 — R5b·W24는 각각 별도 마이그레이션·Codex 승인.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 26개 — 완료 23 · 보류 2 · 진행 중 1</t>
+          <t>총 27개 — 완료 24 · 보류 2 · 진행 중 1</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1799,92 +1799,142 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W23-R5a</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>운영 UX 팩 — 단가 입력·적용단가 표시·발주 문장·이번 발주만 매입처</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>매일 만지는 곳 네 군데를 손봤습니다. ①금액 칸을 누르면 숫자가 전체 선택되고 Enter로 다음 칸으로 넘어갑니다(선행 0 자동 정리). ②단가 관리에서 거래처별 단가·품목 기본 출고단가·실제 적용 단가를 나란히 보여주고, 기본 단가가 있으면 '미등록' 대신 '기본 단가 적용 중'으로 표시합니다. ③매입처 발주 문장 첫 줄에 발주일이 들어가고, 문장을 직접 고칠 수 있으며, 품목을 바꿔도 고친 문장은 유지되고 '문장 다시 만들기'를 눌러야 새로 만들어집니다. ④합산표에서 이번 발주만 다른 매입처로 바꿀 수 있습니다(품목 기본 매입처는 그대로).</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>완벽한 단가표를 먼저 만드는 ERP가 아니라, 오늘 발주를 빠르게 처리하는 도구라는 원칙. 확정 스냅샷·상태 모델·테이블을 건드리지 않고 체감 불편만 없앤다. R4 대시보드보다 앞서 넣을 수 있는 안전 팩.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>R3/0011 커밋(c31ec1f) 후 진행. 마이그레이션·스키마 0. 매입처 override·문장 편집분은 화면 상태 전용(DB·localStorage 저장 안 함).</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>web 184/184(신규 11: aggregate 날짜·override, price-store effective, price-input 정규화) · root 5/5 · build 성공 · tsc 통과 · audit 0 · diff-check clean. 데모 smoke: 파싱 Enter→다음 칸 · 단가 관리 base-only '기본 단가 적용 중' · 계란(미지정)→야채 이번만 재배정→미지정 0·문장 재그룹 · 발주 문장 날짜/편집 유지/다시 만들기 · 회귀(주문 확정·가격 마감 09000→9000·명세서) · 모바일 390px 오버플로 없음 · 콘솔 0. 미커밋 — Codex 검수 대기. 의도적 편차: 단가 관리 Enter=저장 유지(일괄 저장 없어 키보드 저장 경로 보존).</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>web/src/lib/price-input.ts
+docs/superpowers/specs/2026-07-11-order-moa-operations-ux-tax-design.md
+docs/task-prompt-W23-R5a-operational-ux-pack.md
+docs/agent-worklog.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1893,48 +1943,48 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>

<commit_message>
feat: add confirmed order correction flow
</commit_message>
<xml_diff>
--- a/docs/order-moa-progress-tracker.xlsx
+++ b/docs/order-moa-progress-tracker.xlsx
@@ -58,12 +58,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -512,7 +512,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>W23-R5a 운영 UX 팩 구현·검수 완료(마이그레이션 0, web 186/186). 가격 입력 전체선택/Enter·단가 관리 적용 단가 표시·매입처 발주 문장 날짜·편집·이번 발주만 매입처 변경, 거래처·날짜 필터 변경 시 임시 재지정·편집본 초기화까지 됨. 다음 후보: W23-R5b 확정 주문 정정(취소→복사→재확정) / W23-R4 대시보드 오늘 업무 큐 / W24 품목코드·과세구분 — R5b·W24는 각각 별도 마이그레이션·Codex 승인.</t>
+          <t>W23-R4 오늘 업무 큐는 통합 완료. W23-R5b 확정 주문 정정은 코드·0012 초안·자동 검증까지 완료됐고, 사용자 SQL Editor의 0012 적용과 로그인 DB smoke(G1~G12 포함)가 남아 진행 중이다. 원주문 스냅샷 불변·가격 대기 격리·raw_text 삭제 가능 원칙을 유지한다. 다음 후보는 0012 적용 검증 뒤 R5b 통합, 그 다음 W24 품목코드·과세구분(별도 승인)이다.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>총 27개 — 완료 24 · 보류 2 · 진행 중 1</t>
+          <t>총 29개 — 완료 25 · 진행 중 2 · 보류 2</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1849,92 +1849,190 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W23-R4</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>인쇄/명세서 양식 보정</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>보류</t>
+          <t>오늘 업무 대시보드 큐</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>1.5차</t>
+          <t>2차 보강</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+          <t>대시보드가 저장된 주문 상태만 읽어 오늘 할 일을 보여줍니다. 가격 대기는 날짜와 무관하게 모두, 명세서 준비와 매입처 발주는 오늘 주문만 계산하며 취소 주문은 모든 카드에서 제외됩니다.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+          <t>가격 대기와 당일 마감 업무를 첫 화면에서 바로 구분해, 확인·마감·명세서 흐름으로 빠르게 들어가게 한다.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+          <t>완료. 마이그레이션과 새 저장값 없이 기존 주문 상태를 읽기 전용으로 집계한다.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+          <t>root 5/5 · web 195/195 · build · tsc · audit 0 · diff-check clean. 데모 smoke에서 가격 대기/명세서/매입처 발주 카드 수치·직행·모바일 390px을 확인했다.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>docs/delivery-note-print-spec.md</t>
+          <t>web/src/lib/dashboard-queue.ts
+web/src/app/order-list-filter.ts
+docs/agent-worklog.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>W23-R5b</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>확정 주문 정정 — 취소·복사·새 주문 재확정</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>진행 중</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2차 보강</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>최종 확정 주문은 직접 고치지 않고, 정정 확정 때만 원주문을 취소 이력으로 남긴 뒤 품목·수량·단가를 복사한 새 주문을 확정합니다. 가격 대기 주문은 정정 대상이 아니며, 새 주문은 원주문 연결을 보존합니다.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>확정 단가 스냅샷과 기존 거래명세서를 바꾸지 않으면서, 실무 정정을 추적 가능하게 만든다.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>0012_order_correction_link.sql은 아직 미적용. 사용자 SQL Editor에서 적용하고 G1~G12 가드 실측 및 로그인 DB smoke를 마친 뒤에만 완료/통합 판단한다.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>구현 worktree 자동 검증 예정: root npm test · web npm test · build · tsc · audit · diff-check. 0012 미적용 DB는 컬럼 폴백으로 기존 주문 기능을 유지하고 정정 UI를 숨긴다.</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>docs/superpowers/specs/2026-07-12-order-moa-r5b-correction-design.md
+docs/guide-apply-0012-order-correction-link.md
+web/supabase/migrations/0012_order_correction_link.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>인쇄/명세서 양식 보정</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>1.5차</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>거래명세서를 더 실서류답게(공급자/거래처 정보 블록, 규격 칸, 금액 한글 표기 등) 다듬습니다. 인쇄는 계속 브라우저 인쇄창.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>지금 양식도 쓸 수는 있어서 1차 완성 뒤로 미룹니다. PDF 파일 생성은 2차.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>1차 완료(W02~W13). 기준: delivery-note-print-spec.md.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>인쇄 미리보기에서 A4 한 장 정돈 확인, 품목 적을 때 빈행 유지.</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>docs/delivery-note-print-spec.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>엑셀/백업/내보내기</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>1차</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>내보내기(CSV) 절반 완료(2026-07-08): '데이터 내보내기' 화면에서 거래처·매입처·품목별칭·단가·주문 목록을 CSV로 내려받고, 월 합계 화면에서 선택 월 합계를 CSV로 내려받아 보관. 공유 Supabase 쿼터 위험 대비 백업 + 회계사 전달용. 금액은 확정 당시 스냅샷. 가져오기(엑셀 업로드)·전체 zip·JSON 백업은 후순위.</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>공유 DB가 막히기 전에 손에 파일로 데이터를 확보(안전망) + 전용 프로젝트 분리의 첫 단계. 초기 세팅용 엑셀 업로드는 후순위.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>완료 — 기준정보 CRUD(W02~W04·W07) + 저장 주문(W08~W12).</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>데모 실측(2026-07-08): 6종 CSV 다운로드 가로채 내용 확인(escape·BOM·스냅샷 금액). 콤마 포함 메모/품목요약 정상 quoting, CSV 인젝션 방어. 가져오기 검증은 미구현(후순위).</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>web/src/lib/csv-export.ts
 web/src/app/page.tsx
@@ -1943,48 +2041,48 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>2차 보류: 미수금·세금계산서 근거·원가/재고</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>보류</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>2차</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>못 받은 돈(미수금) 체크, 월별 세금계산서 발행 금액 대조, 매입처별 원가 이력, 좁은 재고. 지금은 만들지 않습니다.</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>1차 주문 데이터가 4주 이상 실사용으로 쌓인 뒤에 만들어야 추측이 아닌 설계가 됩니다. 근거 데이터(주문 금액)는 1차부터 이미 보존 중.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>1차+1.5차 완료 + 실사용 4주. OCR/카톡 자동 읽기/이카운트 연동/직접 발행은 별도로 '제외'(착수 금지).</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>착수 시점에 로드맵 2차 선행 조건 재확인.</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>docs/order-moa-expanded-roadmap.md(2차·제외)</t>
         </is>

</xml_diff>